<commit_message>
fixed the strechable chain bug
</commit_message>
<xml_diff>
--- a/src/utils/vis/acm.xlsx
+++ b/src/utils/vis/acm.xlsx
@@ -431,169 +431,169 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>right_ankle_roll_link</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>logo_link</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>left_knee_link</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>right_hip_pitch_link</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>right_shoulder_roll_link</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>left_ankle_roll_link</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>right_wrist_pitch_link</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>right_hip_yaw_link</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>right_elbow_link</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>right_shoulder_pitch_link</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>right_rubber_hand</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>left_ankle_pitch_link</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>torso_link</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>head_link</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>left_hip_yaw_link</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>left_shoulder_pitch_link</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>left_hip_roll_link</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>right_wrist_roll_link</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>left_hip_yaw_link</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>left_ankle_roll_link</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>torso_link</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>logo_link</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>right_hip_yaw_link</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>left_wrist_pitch_link</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>left_wrist_roll_link</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>right_shoulder_yaw_link</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>right_hip_roll_link</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>left_ankle_pitch_link</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>right_wrist_pitch_link</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>right_hip_pitch_link</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>right_shoulder_pitch_link</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>left_wrist_roll_link</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>right_rubber_hand</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>right_elbow_link</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>pelvis_contour_link</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>left_elbow_link</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>left_shoulder_roll_link</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>left_hip_pitch_link</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>right_wrist_yaw_link</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>left_shoulder_yaw_link</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>left_rubber_hand</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>left_wrist_yaw_link</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>right_ankle_pitch_link</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>right_knee_link</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>right_ankle_roll_link</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>right_shoulder_yaw_link</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>left_knee_link</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>left_rubber_hand</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>right_shoulder_roll_link</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>left_hip_pitch_link</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>right_wrist_yaw_link</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>left_hip_roll_link</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>left_shoulder_roll_link</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>left_elbow_link</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>left_shoulder_yaw_link</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>pelvis_contour_link</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>left_shoulder_pitch_link</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>left_wrist_yaw_link</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>right_ankle_pitch_link</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>left_wrist_pitch_link</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>head_link</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>right_wrist_roll_link</t>
+          <t>right_ankle_roll_link</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -612,55 +612,55 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V2" t="n">
         <v>1</v>
       </c>
       <c r="W2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" t="n">
         <v>1</v>
@@ -684,19 +684,19 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>left_hip_yaw_link</t>
+          <t>logo_link</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -706,22 +706,22 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -736,22 +736,22 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
@@ -760,10 +760,10 @@
         <v>1</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X3" t="n">
         <v>0</v>
@@ -772,13 +772,13 @@
         <v>1</v>
       </c>
       <c r="Z3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC3" t="n">
         <v>1</v>
@@ -799,32 +799,32 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>left_ankle_roll_link</t>
+          <t>left_knee_link</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -836,25 +836,25 @@
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="n">
         <v>1</v>
       </c>
       <c r="P4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
@@ -878,7 +878,7 @@
         <v>1</v>
       </c>
       <c r="AA4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
         <v>1</v>
@@ -890,7 +890,7 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF4" t="n">
         <v>1</v>
@@ -902,7 +902,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>torso_link</t>
+          <t>right_hip_pitch_link</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -912,7 +912,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -936,55 +936,55 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
         <v>1</v>
       </c>
       <c r="N5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V5" t="n">
         <v>0</v>
       </c>
       <c r="W5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X5" t="n">
         <v>0</v>
       </c>
       <c r="Y5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1005,14 +1005,14 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>logo_link</t>
+          <t>right_shoulder_roll_link</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
@@ -1033,19 +1033,19 @@
         <v>1</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" t="n">
         <v>1</v>
       </c>
       <c r="N6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O6" t="n">
         <v>1</v>
@@ -1054,43 +1054,43 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" t="n">
         <v>0</v>
       </c>
       <c r="W6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X6" t="n">
         <v>0</v>
       </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD6" t="n">
         <v>1</v>
@@ -1102,23 +1102,23 @@
         <v>1</v>
       </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>right_hip_yaw_link</t>
+          <t>left_ankle_roll_link</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -1130,7 +1130,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
@@ -1139,16 +1139,16 @@
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
         <v>1</v>
@@ -1157,7 +1157,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" t="n">
         <v>1</v>
@@ -1172,13 +1172,13 @@
         <v>1</v>
       </c>
       <c r="V7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W7" t="n">
         <v>1</v>
       </c>
       <c r="X7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y7" t="n">
         <v>1</v>
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="AB7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC7" t="n">
         <v>1</v>
@@ -1199,10 +1199,10 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG7" t="n">
         <v>1</v>
@@ -1211,14 +1211,14 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>right_hip_roll_link</t>
+          <t>right_wrist_pitch_link</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1239,7 +1239,7 @@
         <v>1</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1257,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="P8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" t="n">
         <v>1</v>
@@ -1266,13 +1266,13 @@
         <v>1</v>
       </c>
       <c r="S8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" t="n">
         <v>0</v>
@@ -1281,10 +1281,10 @@
         <v>1</v>
       </c>
       <c r="X8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="n">
         <v>1</v>
@@ -1293,38 +1293,38 @@
         <v>1</v>
       </c>
       <c r="AB8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD8" t="n">
         <v>1</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF8" t="n">
         <v>1</v>
       </c>
       <c r="AG8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>left_ankle_pitch_link</t>
+          <t>right_hip_yaw_link</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1351,7 +1351,7 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
@@ -1363,13 +1363,13 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -1378,50 +1378,50 @@
         <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" t="n">
         <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB9" t="n">
         <v>1</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD9" t="n">
         <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>right_wrist_pitch_link</t>
+          <t>right_elbow_link</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -1433,13 +1433,13 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>1</v>
@@ -1448,7 +1448,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1457,10 +1457,10 @@
         <v>1</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" t="n">
         <v>1</v>
@@ -1469,22 +1469,22 @@
         <v>1</v>
       </c>
       <c r="R10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T10" t="n">
         <v>1</v>
       </c>
       <c r="U10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10" t="n">
         <v>1</v>
@@ -1496,10 +1496,10 @@
         <v>1</v>
       </c>
       <c r="AA10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC10" t="n">
         <v>1</v>
@@ -1520,7 +1520,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>right_hip_pitch_link</t>
+          <t>right_shoulder_pitch_link</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1539,7 +1539,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1548,61 +1548,61 @@
         <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
         <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11" t="n">
         <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" t="n">
         <v>0</v>
       </c>
       <c r="W11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X11" t="n">
         <v>0</v>
       </c>
       <c r="Y11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
         <v>0</v>
       </c>
       <c r="AB11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -1617,17 +1617,17 @@
         <v>1</v>
       </c>
       <c r="AG11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>right_shoulder_pitch_link</t>
+          <t>right_rubber_hand</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C12" t="n">
         <v>1</v>
@@ -1636,10 +1636,10 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
@@ -1654,7 +1654,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1666,7 +1666,7 @@
         <v>1</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
@@ -1675,16 +1675,16 @@
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T12" t="n">
         <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V12" t="n">
         <v>0</v>
@@ -1693,22 +1693,22 @@
         <v>1</v>
       </c>
       <c r="X12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z12" t="n">
         <v>1</v>
       </c>
       <c r="AA12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD12" t="n">
         <v>1</v>
@@ -1720,23 +1720,23 @@
         <v>1</v>
       </c>
       <c r="AG12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>left_wrist_roll_link</t>
+          <t>left_ankle_pitch_link</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="n">
         <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -1745,13 +1745,13 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
         <v>1</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -1766,19 +1766,19 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="n">
         <v>1</v>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>1</v>
@@ -1787,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
         <v>1</v>
@@ -1799,7 +1799,7 @@
         <v>1</v>
       </c>
       <c r="Y13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z13" t="n">
         <v>0</v>
@@ -1811,10 +1811,10 @@
         <v>1</v>
       </c>
       <c r="AC13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE13" t="n">
         <v>1</v>
@@ -1829,26 +1829,26 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>right_rubber_hand</t>
+          <t>torso_link</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
         <v>1</v>
@@ -1857,16 +1857,16 @@
         <v>1</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
@@ -1875,10 +1875,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1896,19 +1896,19 @@
         <v>1</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y14" t="n">
         <v>1</v>
       </c>
       <c r="Z14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="n">
         <v>1</v>
@@ -1932,20 +1932,20 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>right_elbow_link</t>
+          <t>head_link</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
@@ -1960,13 +1960,13 @@
         <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
         <v>1</v>
@@ -1981,7 +1981,7 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1993,16 +1993,16 @@
         <v>1</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y15" t="n">
         <v>1</v>
@@ -2011,7 +2011,7 @@
         <v>1</v>
       </c>
       <c r="AA15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB15" t="n">
         <v>1</v>
@@ -2035,7 +2035,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>right_knee_link</t>
+          <t>left_hip_yaw_link</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2045,10 +2045,10 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
         <v>1</v>
@@ -2057,7 +2057,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>1</v>
@@ -2066,16 +2066,16 @@
         <v>1</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O16" t="n">
         <v>1</v>
@@ -2084,10 +2084,10 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" t="n">
         <v>1</v>
@@ -2102,10 +2102,10 @@
         <v>1</v>
       </c>
       <c r="W16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y16" t="n">
         <v>1</v>
@@ -2114,7 +2114,7 @@
         <v>1</v>
       </c>
       <c r="AA16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB16" t="n">
         <v>1</v>
@@ -2126,7 +2126,7 @@
         <v>1</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
         <v>1</v>
@@ -2138,98 +2138,98 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>right_ankle_roll_link</t>
+          <t>left_shoulder_pitch_link</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S17" t="n">
         <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB17" t="n">
         <v>1</v>
       </c>
       <c r="AC17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF17" t="n">
         <v>1</v>
@@ -2241,23 +2241,23 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>right_shoulder_yaw_link</t>
+          <t>left_hip_roll_link</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
@@ -2266,19 +2266,19 @@
         <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
@@ -2287,10 +2287,10 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -2302,7 +2302,7 @@
         <v>1</v>
       </c>
       <c r="U18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V18" t="n">
         <v>0</v>
@@ -2311,22 +2311,22 @@
         <v>0</v>
       </c>
       <c r="X18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y18" t="n">
         <v>1</v>
       </c>
       <c r="Z18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD18" t="n">
         <v>1</v>
@@ -2344,41 +2344,41 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>left_knee_link</t>
+          <t>right_wrist_roll_link</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
         <v>1</v>
@@ -2414,7 +2414,7 @@
         <v>1</v>
       </c>
       <c r="X19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y19" t="n">
         <v>1</v>
@@ -2426,7 +2426,7 @@
         <v>1</v>
       </c>
       <c r="AB19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC19" t="n">
         <v>1</v>
@@ -2447,7 +2447,7 @@
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>left_rubber_hand</t>
+          <t>left_wrist_pitch_link</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2496,7 +2496,7 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R20" t="n">
         <v>1</v>
@@ -2508,7 +2508,7 @@
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="n">
         <v>1</v>
@@ -2520,7 +2520,7 @@
         <v>1</v>
       </c>
       <c r="Y20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z20" t="n">
         <v>1</v>
@@ -2532,13 +2532,13 @@
         <v>1</v>
       </c>
       <c r="AC20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF20" t="n">
         <v>1</v>
@@ -2550,11 +2550,11 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>right_shoulder_roll_link</t>
+          <t>left_wrist_roll_link</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
         <v>1</v>
@@ -2563,76 +2563,76 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>1</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>1</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P21" t="n">
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S21" t="n">
         <v>1</v>
       </c>
       <c r="T21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W21" t="n">
         <v>1</v>
       </c>
       <c r="X21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="n">
         <v>1</v>
       </c>
       <c r="AB21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC21" t="n">
         <v>0</v>
@@ -2641,7 +2641,7 @@
         <v>1</v>
       </c>
       <c r="AE21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF21" t="n">
         <v>1</v>
@@ -2653,14 +2653,14 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>left_hip_pitch_link</t>
+          <t>right_shoulder_yaw_link</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
         <v>1</v>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -2696,13 +2696,13 @@
         <v>1</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P22" t="n">
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -2714,7 +2714,7 @@
         <v>1</v>
       </c>
       <c r="U22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -2726,7 +2726,7 @@
         <v>0</v>
       </c>
       <c r="Y22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z22" t="n">
         <v>1</v>
@@ -2738,7 +2738,7 @@
         <v>0</v>
       </c>
       <c r="AC22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD22" t="n">
         <v>1</v>
@@ -2750,29 +2750,29 @@
         <v>1</v>
       </c>
       <c r="AG22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>right_wrist_yaw_link</t>
+          <t>right_hip_roll_link</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" t="n">
         <v>1</v>
@@ -2781,13 +2781,13 @@
         <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
         <v>1</v>
@@ -2796,16 +2796,16 @@
         <v>1</v>
       </c>
       <c r="N23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2832,10 +2832,10 @@
         <v>1</v>
       </c>
       <c r="Z23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB23" t="n">
         <v>1</v>
@@ -2850,16 +2850,16 @@
         <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>left_hip_roll_link</t>
+          <t>pelvis_contour_link</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2878,10 +2878,10 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
@@ -2893,34 +2893,34 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" t="n">
         <v>1</v>
       </c>
       <c r="N24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T24" t="n">
         <v>1</v>
       </c>
       <c r="U24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -2935,10 +2935,10 @@
         <v>0</v>
       </c>
       <c r="Z24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB24" t="n">
         <v>1</v>
@@ -2956,13 +2956,13 @@
         <v>1</v>
       </c>
       <c r="AG24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>left_shoulder_roll_link</t>
+          <t>left_elbow_link</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -2975,31 +2975,31 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" t="n">
         <v>1</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
         <v>1</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" t="n">
         <v>1</v>
@@ -3011,7 +3011,7 @@
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
         <v>1</v>
@@ -3020,13 +3020,13 @@
         <v>1</v>
       </c>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W25" t="n">
         <v>1</v>
@@ -3041,10 +3041,10 @@
         <v>0</v>
       </c>
       <c r="AA25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC25" t="n">
         <v>0</v>
@@ -3053,7 +3053,7 @@
         <v>1</v>
       </c>
       <c r="AE25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF25" t="n">
         <v>1</v>
@@ -3065,23 +3065,23 @@
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>left_elbow_link</t>
+          <t>left_shoulder_roll_link</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>1</v>
@@ -3096,7 +3096,7 @@
         <v>1</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
         <v>1</v>
@@ -3105,7 +3105,7 @@
         <v>0</v>
       </c>
       <c r="N26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O26" t="n">
         <v>1</v>
@@ -3114,10 +3114,10 @@
         <v>1</v>
       </c>
       <c r="Q26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
         <v>1</v>
@@ -3126,16 +3126,16 @@
         <v>1</v>
       </c>
       <c r="U26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V26" t="n">
         <v>1</v>
       </c>
       <c r="W26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y26" t="n">
         <v>0</v>
@@ -3147,19 +3147,19 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE26" t="n">
         <v>1</v>
       </c>
       <c r="AF26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG26" t="n">
         <v>1</v>
@@ -3168,23 +3168,23 @@
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>left_shoulder_yaw_link</t>
+          <t>left_hip_pitch_link</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>1</v>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G27" t="n">
         <v>1</v>
@@ -3193,34 +3193,34 @@
         <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
         <v>0</v>
       </c>
       <c r="N27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>1</v>
@@ -3235,13 +3235,13 @@
         <v>0</v>
       </c>
       <c r="W27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z27" t="n">
         <v>0</v>
@@ -3250,19 +3250,19 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE27" t="n">
         <v>1</v>
       </c>
       <c r="AF27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG27" t="n">
         <v>1</v>
@@ -3271,38 +3271,38 @@
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>pelvis_contour_link</t>
+          <t>right_wrist_yaw_link</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -3323,16 +3323,16 @@
         <v>1</v>
       </c>
       <c r="R28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T28" t="n">
         <v>1</v>
       </c>
       <c r="U28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V28" t="n">
         <v>0</v>
@@ -3344,19 +3344,19 @@
         <v>1</v>
       </c>
       <c r="Y28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
       </c>
       <c r="AC28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD28" t="n">
         <v>1</v>
@@ -3368,13 +3368,13 @@
         <v>1</v>
       </c>
       <c r="AG28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>left_shoulder_pitch_link</t>
+          <t>left_shoulder_yaw_link</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -3390,16 +3390,16 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="n">
         <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -3408,10 +3408,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
         <v>1</v>
@@ -3423,22 +3423,22 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S29" t="n">
         <v>1</v>
       </c>
       <c r="T29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W29" t="n">
         <v>1</v>
@@ -3456,7 +3456,7 @@
         <v>0</v>
       </c>
       <c r="AB29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC29" t="n">
         <v>0</v>
@@ -3465,19 +3465,19 @@
         <v>1</v>
       </c>
       <c r="AE29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>left_wrist_yaw_link</t>
+          <t>left_rubber_hand</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -3514,7 +3514,7 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N30" t="n">
         <v>1</v>
@@ -3526,7 +3526,7 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>1</v>
@@ -3535,7 +3535,7 @@
         <v>1</v>
       </c>
       <c r="T30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U30" t="n">
         <v>1</v>
@@ -3553,10 +3553,10 @@
         <v>1</v>
       </c>
       <c r="Z30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB30" t="n">
         <v>1</v>
@@ -3568,10 +3568,10 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG30" t="n">
         <v>1</v>
@@ -3580,17 +3580,17 @@
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>right_ankle_pitch_link</t>
+          <t>left_wrist_yaw_link</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" t="n">
         <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
@@ -3599,13 +3599,13 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
         <v>1</v>
@@ -3626,10 +3626,10 @@
         <v>1</v>
       </c>
       <c r="P31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
@@ -3638,10 +3638,10 @@
         <v>1</v>
       </c>
       <c r="T31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V31" t="n">
         <v>1</v>
@@ -3653,7 +3653,7 @@
         <v>1</v>
       </c>
       <c r="Y31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z31" t="n">
         <v>1</v>
@@ -3665,10 +3665,10 @@
         <v>1</v>
       </c>
       <c r="AC31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
@@ -3683,11 +3683,11 @@
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>left_wrist_pitch_link</t>
+          <t>right_ankle_pitch_link</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" t="n">
         <v>1</v>
@@ -3702,13 +3702,13 @@
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
       </c>
       <c r="I32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
         <v>1</v>
@@ -3750,7 +3750,7 @@
         <v>1</v>
       </c>
       <c r="W32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X32" t="n">
         <v>1</v>
@@ -3759,19 +3759,19 @@
         <v>1</v>
       </c>
       <c r="Z32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB32" t="n">
         <v>1</v>
       </c>
       <c r="AC32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE32" t="n">
         <v>1</v>
@@ -3780,17 +3780,17 @@
         <v>0</v>
       </c>
       <c r="AG32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>head_link</t>
+          <t>right_knee_link</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" t="n">
         <v>1</v>
@@ -3802,25 +3802,25 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="n">
         <v>1</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M33" t="n">
         <v>1</v>
@@ -3850,13 +3850,13 @@
         <v>1</v>
       </c>
       <c r="V33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y33" t="n">
         <v>1</v>
@@ -3868,10 +3868,10 @@
         <v>1</v>
       </c>
       <c r="AB33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD33" t="n">
         <v>1</v>
@@ -3880,7 +3880,7 @@
         <v>1</v>
       </c>
       <c r="AF33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG33" t="n">
         <v>0</v>

</xml_diff>